<commit_message>
still updating team info
</commit_message>
<xml_diff>
--- a/ressources/people_location.xlsx
+++ b/ressources/people_location.xlsx
@@ -1,20 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mpetera\Documents\MyDrive\Workspace\ScriptR\GIT\W4MwebGHpage\ressources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3A03E3D-BF1A-49AD-815B-2D46353C9710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="32895" yWindow="3390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Feuil1"/>
+    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="89">
   <si>
     <t>long</t>
   </si>
@@ -40,12 +62,6 @@
     <t>country</t>
   </si>
   <si>
-    <t>3.01629</t>
-  </si>
-  <si>
-    <t>45.71213</t>
-  </si>
-  <si>
     <t>Binta Diémé</t>
   </si>
   <si>
@@ -55,21 +71,12 @@
     <t>Route de Theix</t>
   </si>
   <si>
-    <t>Saint-Genês-Champanelle</t>
-  </si>
-  <si>
     <t>France</t>
   </si>
   <si>
     <t>Charlotte Joly</t>
   </si>
   <si>
-    <t>1.3749738661049271</t>
-  </si>
-  <si>
-    <t>43.60249300145284</t>
-  </si>
-  <si>
     <t>Cécile Canlet</t>
   </si>
   <si>
@@ -82,12 +89,6 @@
     <t>Toulouse</t>
   </si>
   <si>
-    <t>4.3961032004916145</t>
-  </si>
-  <si>
-    <t>50.818092092542436</t>
-  </si>
-  <si>
     <t>Cédric Delporte</t>
   </si>
   <si>
@@ -121,24 +122,6 @@
     <t>Brétigny-sur-Orge</t>
   </si>
   <si>
-    <t>2.1767607</t>
-  </si>
-  <si>
-    <t>48.765236</t>
-  </si>
-  <si>
-    <t>Eric Venot</t>
-  </si>
-  <si>
-    <t>GABI</t>
-  </si>
-  <si>
-    <t>Domaine de Vilvert</t>
-  </si>
-  <si>
-    <t>Jouy-en-josas</t>
-  </si>
-  <si>
     <t>2.1487911556484773</t>
   </si>
   <si>
@@ -151,15 +134,9 @@
     <t>CEA</t>
   </si>
   <si>
-    <t>Saclay</t>
-  </si>
-  <si>
     <t>Florence Souard</t>
   </si>
   <si>
-    <t>Franck Giacomoni</t>
-  </si>
-  <si>
     <t>-3.98708</t>
   </si>
   <si>
@@ -193,33 +170,15 @@
     <t>Czech Republic</t>
   </si>
   <si>
-    <t>1.0706026520893674</t>
-  </si>
-  <si>
-    <t>49.45800142743788</t>
-  </si>
-  <si>
     <t>Isabelle Schmitz</t>
   </si>
   <si>
     <t>PBS</t>
   </si>
   <si>
-    <t>Bd Maurice de Broglie</t>
-  </si>
-  <si>
     <t>Mont Saint Aignan</t>
   </si>
   <si>
-    <t>-1.52532</t>
-  </si>
-  <si>
-    <t>47.28945</t>
-  </si>
-  <si>
-    <t>Julien Saint-Vanne</t>
-  </si>
-  <si>
     <t>LABERCA</t>
   </si>
   <si>
@@ -244,12 +203,6 @@
     <t>Nils Paulhe</t>
   </si>
   <si>
-    <t>-1.9311562376160851</t>
-  </si>
-  <si>
-    <t>52.44991582676665</t>
-  </si>
-  <si>
     <t>Ralf Weber</t>
   </si>
   <si>
@@ -268,12 +221,6 @@
     <t>United-Kingdom</t>
   </si>
   <si>
-    <t>-1.792899</t>
-  </si>
-  <si>
-    <t>48.1090675</t>
-  </si>
-  <si>
     <t>Sylvain Chéreau</t>
   </si>
   <si>
@@ -299,14 +246,70 @@
   </si>
   <si>
     <t>Fance</t>
+  </si>
+  <si>
+    <t>3.0734329223632812</t>
+  </si>
+  <si>
+    <t>45.7717170715332</t>
+  </si>
+  <si>
+    <t>Etienne Jules</t>
+  </si>
+  <si>
+    <t>Saint-Genès-Champanelle</t>
+  </si>
+  <si>
+    <t>1.071152225809878</t>
+  </si>
+  <si>
+    <t>49.459541854137356</t>
+  </si>
+  <si>
+    <t>Place Emile Blondel, Batiment CURIB</t>
+  </si>
+  <si>
+    <t>48.10940456692299</t>
+  </si>
+  <si>
+    <t>-1.7932468272979607</t>
+  </si>
+  <si>
+    <t>1.373884</t>
+  </si>
+  <si>
+    <t>43.6022883</t>
+  </si>
+  <si>
+    <t>Centre CEA Paris-Saclay</t>
+  </si>
+  <si>
+    <t>Gif-sur-Yvette</t>
+  </si>
+  <si>
+    <t>4.3823</t>
+  </si>
+  <si>
+    <t>Axelle Bourez</t>
+  </si>
+  <si>
+    <t>49.1936</t>
+  </si>
+  <si>
+    <t>16.6033</t>
+  </si>
+  <si>
+    <t>52.4508</t>
+  </si>
+  <si>
+    <t>-1.9305</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -344,6 +347,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -372,65 +382,63 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+  <cellXfs count="18">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -441,10 +449,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -482,71 +490,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -574,7 +582,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -597,11 +605,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -610,13 +618,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -626,7 +634,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -635,7 +643,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -644,7 +652,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -652,10 +660,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -720,27 +728,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="14" width="30.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="14" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="9.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="14" width="40.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="15" width="7.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="14" width="15.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="14" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="30.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.5703125" style="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" style="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -769,575 +776,553 @@
       <c r="J1" s="1"/>
       <c r="K1" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="8">
+        <v>1050</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="4">
-        <v>63122</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="F3" s="4">
         <v>63122</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
+    <row r="4" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>71</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="6">
-        <v>31027</v>
+        <v>9</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="4">
+        <v>63122</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="8">
-        <v>1050</v>
+        <v>14</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="6">
+        <v>31027</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>30</v>
+    <row r="6" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>83</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="4">
-        <v>91220</v>
+        <v>18</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="8">
+        <v>1050</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="F7" s="4">
-        <v>78350</v>
+        <v>91220</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75" customFormat="1" s="9">
+    <row r="8" spans="1:11" s="9" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="10"/>
+        <v>31</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F8" s="10">
+        <v>91190</v>
+      </c>
       <c r="G8" s="3" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>22</v>
+        <v>83</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F9" s="8">
         <v>1050</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="1" t="s">
+    <row r="10" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="E10" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F10" s="4">
         <v>63122</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="F11" s="4">
-        <v>58965</v>
+        <v>29680</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="12">
-        <v>16.571671383796325</v>
-      </c>
-      <c r="B12" s="12">
-        <v>49.17879303863339</v>
+    <row r="12" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>85</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="F12" s="2">
         <v>62500</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F13" s="4">
-        <v>76821</v>
+        <v>76130</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>66</v>
+    <row r="14" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>80</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>69</v>
+        <v>51</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="F14" s="4">
-        <v>44307</v>
+        <v>31300</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>17</v>
+    <row r="15" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>71</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="4">
+        <v>63122</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F15" s="4">
-        <v>31300</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="H15" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="1" t="s">
+    <row r="16" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="E16" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F16" s="4">
         <v>63122</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="1" t="s">
-        <v>8</v>
+    <row r="17" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="17" t="s">
+        <v>88</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>11</v>
+        <v>56</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="4">
-        <v>63122</v>
+        <v>57</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>77</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>81</v>
+        <v>63</v>
+      </c>
+      <c r="F18" s="4">
+        <v>35653</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F19" s="4">
-        <v>35650</v>
+        <v>81</v>
+      </c>
+      <c r="F19" s="2">
+        <v>91190</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="1"/>
+        <v>47</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="4">
+        <v>44307</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="H20" s="1" t="s">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="F21" s="4">
-        <v>44307</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>